<commit_message>
ARCH NIH, and Child_ECHO_ID
</commit_message>
<xml_diff>
--- a/Data Pull/Shipp/R01 Dairy Data Table.xlsx
+++ b/Data Pull/Shipp/R01 Dairy Data Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://michiganstate-my.sharepoint.com/personal/tianjiah_msu_edu/Documents/Data Manager/Data-Manager/Data Pull/Shipp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{D1F4D2BB-7FC3-459B-9BDB-B5E80F70264D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{603D5A61-F5E0-42A6-A276-E09F0A63032A}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="13_ncr:1_{D1F4D2BB-7FC3-459B-9BDB-B5E80F70264D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C81E76D-DAD5-47E6-90CE-6FC68B08ACF1}"/>
   <bookViews>
-    <workbookView xWindow="9700" yWindow="-21600" windowWidth="19380" windowHeight="20970" xr2:uid="{95CC1F47-BD34-4B62-B12F-8961E3FDFA8B}"/>
+    <workbookView xWindow="-9350" yWindow="-21040" windowWidth="23260" windowHeight="12460" xr2:uid="{95CC1F47-BD34-4B62-B12F-8961E3FDFA8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -547,24 +547,42 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -588,24 +606,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1032,23 +1032,23 @@
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="39"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -1060,19 +1060,19 @@
       <c r="B2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="42"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="41" t="s">
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="43"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="30"/>
       <c r="L2" s="8"/>
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1089,7 +1089,7 @@
       <c r="E3" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="31" t="s">
+      <c r="F3" s="37" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="7" t="s">
@@ -1110,7 +1110,7 @@
       <c r="C4" s="24"/>
       <c r="D4" s="24"/>
       <c r="E4" s="24"/>
-      <c r="F4" s="32"/>
+      <c r="F4" s="38"/>
       <c r="G4" s="6" t="s">
         <v>26</v>
       </c>
@@ -1132,34 +1132,34 @@
         <v>1</v>
       </c>
       <c r="B5" s="13">
-        <v>1027</v>
+        <v>999</v>
       </c>
       <c r="C5" s="13">
+        <v>610</v>
+      </c>
+      <c r="D5" s="14">
+        <v>136</v>
+      </c>
+      <c r="E5" s="17">
         <v>598</v>
       </c>
-      <c r="D5" s="14">
-        <v>133</v>
-      </c>
-      <c r="E5" s="17">
-        <v>605</v>
-      </c>
       <c r="F5" s="17">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="G5" s="17">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="H5" s="17">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="I5" s="17">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="J5" s="17">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="K5" s="17">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -1167,13 +1167,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="13">
-        <v>409</v>
+        <v>371</v>
       </c>
       <c r="C6" s="13">
         <v>0</v>
       </c>
       <c r="D6" s="13">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E6" s="21" t="s">
         <v>33</v>
@@ -1190,10 +1190,10 @@
       <c r="I6" s="20">
         <v>9</v>
       </c>
-      <c r="J6" s="44" t="s">
+      <c r="J6" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="44"/>
+      <c r="K6" s="31"/>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
@@ -1201,40 +1201,40 @@
       </c>
       <c r="B7" s="13">
         <f t="shared" ref="B7:G7" si="0">B5+B6</f>
-        <v>1436</v>
+        <v>1370</v>
       </c>
       <c r="C7" s="13">
         <f t="shared" si="0"/>
-        <v>598</v>
+        <v>610</v>
       </c>
       <c r="D7" s="13">
         <f t="shared" si="0"/>
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E7" s="17">
-        <v>605</v>
+        <v>598</v>
       </c>
       <c r="F7" s="13">
         <f t="shared" si="0"/>
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="G7" s="13">
         <f t="shared" si="0"/>
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="H7" s="13">
         <f>H5+H6</f>
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="I7" s="13">
         <f>I5+I6</f>
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="J7" s="13">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="K7" s="13">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
@@ -1244,23 +1244,23 @@
       <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
-      <c r="P10" s="40"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="27"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
@@ -1269,66 +1269,66 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="25" t="s">
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="27"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
+      <c r="L11" s="33"/>
+      <c r="M11" s="33"/>
+      <c r="N11" s="33"/>
+      <c r="O11" s="34"/>
     </row>
     <row r="12" spans="1:21" s="1" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
-      <c r="B12" s="30" t="s">
+      <c r="B12" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="25" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="30" t="s">
+      <c r="E12" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30" t="s">
+      <c r="F12" s="25"/>
+      <c r="G12" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30" t="s">
+      <c r="H12" s="25"/>
+      <c r="I12" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="J12" s="30" t="s">
+      <c r="J12" s="25" t="s">
         <v>8</v>
       </c>
       <c r="K12" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="L12" s="30" t="s">
+      <c r="L12" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30" t="s">
+      <c r="M12" s="25"/>
+      <c r="N12" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="O12" s="30"/>
+      <c r="O12" s="25"/>
     </row>
     <row r="13" spans="1:21" s="1" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30"/>
+      <c r="B13" s="25"/>
+      <c r="C13" s="25"/>
       <c r="D13" s="9" t="s">
         <v>26</v>
       </c>
@@ -1344,8 +1344,8 @@
       <c r="H13" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
       <c r="K13" s="9" t="s">
         <v>26</v>
       </c>
@@ -1367,46 +1367,46 @@
         <v>1</v>
       </c>
       <c r="B14" s="16">
-        <v>1027</v>
+        <v>999</v>
       </c>
       <c r="C14" s="16">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D14" s="16">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E14" s="16">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="F14" s="16">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="G14" s="16">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="H14" s="16">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="I14" s="14">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J14" s="16">
         <v>24</v>
       </c>
       <c r="K14" s="16">
+        <v>32</v>
+      </c>
+      <c r="L14" s="16">
+        <v>111</v>
+      </c>
+      <c r="M14" s="16">
         <v>30</v>
       </c>
-      <c r="L14" s="16">
-        <v>108</v>
-      </c>
-      <c r="M14" s="16">
-        <v>28</v>
-      </c>
       <c r="N14" s="16">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="O14" s="14">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
@@ -1416,79 +1416,79 @@
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
-      <c r="O17" s="39"/>
-      <c r="P17" s="39"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="26"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="16"/>
       <c r="B18" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="34" t="s">
+      <c r="D18" s="41"/>
+      <c r="E18" s="42"/>
+      <c r="F18" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="36"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
+      <c r="K18" s="42"/>
     </row>
     <row r="19" spans="1:16" s="2" customFormat="1" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
-      <c r="B19" s="33" t="s">
+      <c r="B19" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="D19" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="33" t="s">
+      <c r="E19" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="F19" s="37" t="s">
+      <c r="F19" s="43" t="s">
         <v>8</v>
       </c>
       <c r="G19" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="H19" s="33" t="s">
+      <c r="H19" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="I19" s="33"/>
-      <c r="J19" s="33" t="s">
+      <c r="I19" s="39"/>
+      <c r="J19" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="K19" s="33"/>
+      <c r="K19" s="39"/>
     </row>
     <row r="20" spans="1:16" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="38"/>
+      <c r="B20" s="39"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="44"/>
       <c r="G20" s="18" t="s">
         <v>26</v>
       </c>
@@ -1509,43 +1509,43 @@
       <c r="A21" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B21" s="16">
-        <v>1027</v>
+      <c r="B21" s="17">
+        <v>999</v>
       </c>
       <c r="C21" s="23">
-        <v>736</v>
+        <v>749</v>
       </c>
       <c r="D21" s="14">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="E21" s="16">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="F21" s="16">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="G21" s="16">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="H21" s="16">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="I21" s="16">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="J21" s="16">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="K21" s="16">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B22" s="16">
-        <v>409</v>
+      <c r="B22" s="17">
+        <v>371</v>
       </c>
       <c r="C22" s="16">
         <v>0</v>
@@ -1554,69 +1554,86 @@
         <v>0</v>
       </c>
       <c r="E22" s="16">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F22" s="16">
-        <v>3</v>
+        <v>43</v>
       </c>
       <c r="G22" s="16">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H22" s="16">
         <v>27</v>
       </c>
       <c r="I22" s="16">
-        <v>60</v>
-      </c>
-      <c r="J22" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="J22" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="K22" s="29"/>
+      <c r="K22" s="36"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B23" s="16">
-        <f>B21+B22</f>
-        <v>1436</v>
+      <c r="B23" s="17">
+        <f t="shared" ref="B23" si="1">B21+B22</f>
+        <v>1370</v>
       </c>
       <c r="C23" s="16">
-        <v>75</v>
+        <v>749</v>
       </c>
       <c r="D23" s="16">
         <f>D21+D22</f>
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="E23" s="16">
         <f>E21+E22</f>
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="F23" s="16">
         <f>F21+F22</f>
-        <v>124</v>
+        <v>167</v>
       </c>
       <c r="G23" s="16">
         <f>G21+G22</f>
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="H23" s="17">
-        <f t="shared" ref="H23:I23" si="1">H21+H22</f>
-        <v>498</v>
+        <f t="shared" ref="H23:I23" si="2">H21+H22</f>
+        <v>506</v>
       </c>
       <c r="I23" s="17">
-        <f t="shared" si="1"/>
-        <v>321</v>
+        <f t="shared" si="2"/>
+        <v>326</v>
       </c>
       <c r="J23" s="16">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="K23" s="16">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B17:P17"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="F18:K18"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="C18:E18"/>
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="C12:C13"/>
@@ -1633,23 +1650,6 @@
     <mergeCell ref="I11:O11"/>
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="G12:H12"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="F18:K18"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="B17:P17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>